<commit_message>
pagina com os slides v18: momento 4 em momento-4.md e aviso de dados ficticios dentro da planilha e do fechamento
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos/kit-parte-1-exemplo-1/arquivos/fechamento-trimestral-2025.xlsx
+++ b/arquivos/kit-parte-1-exemplo-1/arquivos/fechamento-trimestral-2025.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -586,6 +586,13 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Observação: Dados fictícios, criados para o curso IA com Claude (IEL Ceará). Nenhum dado de organização real foi usado.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
pagina sem o aviso de dados ficticios dentro dos arquivos do kit (planilha, fechamento, pessoas, ficha, reuniao bruta, design system)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos/kit-parte-1-exemplo-1/arquivos/fechamento-trimestral-2025.xlsx
+++ b/arquivos/kit-parte-1-exemplo-1/arquivos/fechamento-trimestral-2025.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -586,13 +586,6 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Observação: Dados fictícios, criados para o curso IA com Claude (IEL Ceará). Nenhum dado de organização real foi usado.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
pagina com os slides v20: pratica 1 revista, fechamento sem observacoes contraditorias, como usar sem kit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos/kit-parte-1-exemplo-1/arquivos/fechamento-trimestral-2025.xlsx
+++ b/arquivos/kit-parte-1-exemplo-1/arquivos/fechamento-trimestral-2025.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>duas unidades entraram no meio do trimestre</t>
+          <t>sem ocorrencias</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>concentracao de atividade no fechamento do semestre</t>
+          <t>sem ocorrencias</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>atividade remanejada da unidade Norte</t>
+          <t>ultimo lancamento em 18/12, antes do recesso de fim de ano</t>
         </is>
       </c>
     </row>

</xml_diff>